<commit_message>
feat(reservation): hoan thien 3 tinh nang in an Booking theo mau thuc te (Dong 346, 347, 348)
- Dong 346 (In confirm):
  + Menu toolbar 2 cap Hien gia / Khong hien gia -> In xac nhan dat phong VN & ENG.
  + Mac dinh in tong tien = tong booking.
  + Modal chon dich vu in gom ca Sales va Le tan post (service_bills) de in du cong no.
- Dong 347 (In phieu dang ky khach - Registration Card):
  + Tuy chon Hien gia / Khong hien gia tai Action Dock ben phai.
  + Ho tro in theo phong duoc tick chon hoac toan bo booking.
  + Mau in chuan bang phong, dieu khoan 3 thu tieng (Viet - Anh - Nga) va 3 chu ky.
- Dong 348 (In hoa don tam tinh - Pro-forma Invoice):
  + Menu xo 4 lua chon: In tat ca, In tien phong, In dich vu, Chon dich vu in.
  + Mau Bang ke dich vu / INVOICE chi tiet theo ngay, tien coc, so tien bang chu va lich su thanh toan.
- Dong bo mau in kho A4 truc quan khop cac file Excel tai D:\PMS\MAU IN.
</commit_message>
<xml_diff>
--- a/file word can len plan/Checklist_nghiem_thu_PMS_5_Dot1_v6.xlsx
+++ b/file word can len plan/Checklist_nghiem_thu_PMS_5_Dot1_v6.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="29868" windowHeight="13320" activeTab="3"/>
+    <workbookView windowWidth="29868" windowHeight="13320" activeTab="4"/>
   </bookViews>
   <sheets>
     <sheet name="Lễ tân" sheetId="1" r:id="rId1"/>
@@ -46,7 +46,7 @@
     <t>CHECKLIST NGHIỆM THU PMS — LỄ TÂN</t>
   </si>
   <si>
-    <t>Ngày đánh giá: 09/10/2026 | HKT1 | Ngày nghiệp vụ: 30/08/2026 | Cột Đáp ứng dành cho khách hàng</t>
+    <t xml:space="preserve">Ngày đánh giá: 12/10/2026 </t>
   </si>
   <si>
     <t>Xanh: đạt trong phạm vi ghi rõ | Vàng: đạt một phần | Đỏ: chưa đạt | Xám: chưa kiểm thử</t>
@@ -58,10 +58,10 @@
     <t>Mô tả</t>
   </si>
   <si>
-    <t>Đáp ứng</t>
-  </si>
-  <si>
-    <t>Đánh giá cá nhân</t>
+    <t>Đánh giá từ PMS</t>
+  </si>
+  <si>
+    <t>Đánh giá từ Ringnet</t>
   </si>
   <si>
     <t>Lễ tân

</xml_diff>